<commit_message>
Save local changes before history cleanup
</commit_message>
<xml_diff>
--- a/reconcile/storage/input/inst_canon.xlsx
+++ b/reconcile/storage/input/inst_canon.xlsx
@@ -3633,7 +3633,11 @@
           <t>gravithy</t>
         </is>
       </c>
-      <c r="B220" t="inlineStr"/>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>FR</t>
+        </is>
+      </c>
       <c r="C220" t="inlineStr">
         <is>
           <t>Gravithy</t>
@@ -3895,7 +3899,11 @@
           <t>hydnum steel</t>
         </is>
       </c>
-      <c r="B238" t="inlineStr"/>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
       <c r="C238" t="inlineStr">
         <is>
           <t>Hydnum Steel</t>
@@ -10407,7 +10415,11 @@
           <t>saarstahl</t>
         </is>
       </c>
-      <c r="B686" t="inlineStr"/>
+      <c r="B686" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
       <c r="C686" t="inlineStr">
         <is>
           <t>Saarstahl</t>
@@ -10756,7 +10768,11 @@
           <t>stegra</t>
         </is>
       </c>
-      <c r="B711" t="inlineStr"/>
+      <c r="B711" t="inlineStr">
+        <is>
+          <t>SE</t>
+        </is>
+      </c>
       <c r="C711" t="inlineStr">
         <is>
           <t>Stegra</t>
@@ -11064,7 +11080,7 @@
       </c>
       <c r="C732" t="inlineStr">
         <is>
-          <t>London Electric Vehicle Company</t>
+          <t>LEVC</t>
         </is>
       </c>
     </row>

</xml_diff>